<commit_message>
Sync public webpage data
</commit_message>
<xml_diff>
--- a/forecast-results/河北电网披露及电价预估数据-20260728.xlsx
+++ b/forecast-results/河北电网披露及电价预估数据-20260728.xlsx
@@ -6979,9 +6979,15 @@
       <c r="C2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="13" t="n"/>
-      <c r="E2" s="13" t="n"/>
-      <c r="F2" s="13" t="n"/>
+      <c r="D2" s="13" t="n">
+        <v>413.71</v>
+      </c>
+      <c r="E2" s="13" t="n">
+        <v>410</v>
+      </c>
+      <c r="F2" s="13" t="n">
+        <v>430</v>
+      </c>
       <c r="G2" s="23" t="n">
         <v>414.0154189840235</v>
       </c>
@@ -7014,9 +7020,15 @@
       <c r="C3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="13" t="n"/>
-      <c r="E3" s="13" t="n"/>
-      <c r="F3" s="13" t="n"/>
+      <c r="D3" s="13" t="n">
+        <v>413.71</v>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>410</v>
+      </c>
+      <c r="F3" s="13" t="n">
+        <v>430</v>
+      </c>
       <c r="G3" s="23" t="n">
         <v>413.3590411300846</v>
       </c>
@@ -7049,9 +7061,15 @@
       <c r="C4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="13" t="n"/>
-      <c r="E4" s="13" t="n"/>
-      <c r="F4" s="13" t="n"/>
+      <c r="D4" s="13" t="n">
+        <v>413.71</v>
+      </c>
+      <c r="E4" s="13" t="n">
+        <v>410</v>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>430</v>
+      </c>
       <c r="G4" s="23" t="n">
         <v>413.7218250467544</v>
       </c>
@@ -7084,9 +7102,15 @@
       <c r="C5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="13" t="n"/>
-      <c r="E5" s="13" t="n"/>
-      <c r="F5" s="13" t="n"/>
+      <c r="D5" s="13" t="n">
+        <v>413.71</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>410</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>430</v>
+      </c>
       <c r="G5" s="23" t="n">
         <v>409.8772754828624</v>
       </c>
@@ -7119,9 +7143,15 @@
       <c r="C6" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="13" t="n"/>
-      <c r="E6" s="13" t="n"/>
-      <c r="F6" s="13" t="n"/>
+      <c r="D6" s="13" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>422.49</v>
+      </c>
       <c r="G6" s="23" t="n">
         <v>422.9425794462696</v>
       </c>
@@ -7154,9 +7184,15 @@
       <c r="C7" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="13" t="n"/>
-      <c r="E7" s="13" t="n"/>
-      <c r="F7" s="13" t="n"/>
+      <c r="D7" s="13" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="E7" s="13" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>422.49</v>
+      </c>
       <c r="G7" s="23" t="n">
         <v>414.935525424019</v>
       </c>
@@ -7189,9 +7225,15 @@
       <c r="C8" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="13" t="n"/>
-      <c r="E8" s="13" t="n"/>
-      <c r="F8" s="13" t="n"/>
+      <c r="D8" s="13" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="E8" s="13" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="F8" s="13" t="n">
+        <v>422.49</v>
+      </c>
       <c r="G8" s="23" t="n">
         <v>412.5559100420316</v>
       </c>
@@ -7224,9 +7266,15 @@
       <c r="C9" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="13" t="n"/>
-      <c r="E9" s="13" t="n"/>
-      <c r="F9" s="13" t="n"/>
+      <c r="D9" s="13" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>422.49</v>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>422.49</v>
+      </c>
       <c r="G9" s="23" t="n">
         <v>411.861803409182</v>
       </c>
@@ -7259,9 +7307,15 @@
       <c r="C10" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="13" t="n"/>
-      <c r="E10" s="13" t="n"/>
-      <c r="F10" s="13" t="n"/>
+      <c r="D10" s="13" t="n">
+        <v>402.91</v>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="F10" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G10" s="23" t="n">
         <v>406.0639989264581</v>
       </c>
@@ -7294,9 +7348,15 @@
       <c r="C11" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
+      <c r="D11" s="13" t="n">
+        <v>402.91</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G11" s="23" t="n">
         <v>399.2138582130146</v>
       </c>
@@ -7329,9 +7389,15 @@
       <c r="C12" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
+      <c r="D12" s="13" t="n">
+        <v>402.91</v>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G12" s="23" t="n">
         <v>394.1766358586004</v>
       </c>
@@ -7364,9 +7430,15 @@
       <c r="C13" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
+      <c r="D13" s="13" t="n">
+        <v>402.91</v>
+      </c>
+      <c r="E13" s="13" t="n">
+        <v>400</v>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G13" s="23" t="n">
         <v>391.4129338126875</v>
       </c>
@@ -7399,9 +7471,15 @@
       <c r="C14" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D14" s="13" t="n"/>
-      <c r="E14" s="13" t="n"/>
-      <c r="F14" s="13" t="n"/>
+      <c r="D14" s="13" t="n">
+        <v>394</v>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>392</v>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G14" s="23" t="n">
         <v>391.1524579304986</v>
       </c>
@@ -7434,9 +7512,15 @@
       <c r="C15" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="13" t="n"/>
-      <c r="E15" s="13" t="n"/>
-      <c r="F15" s="13" t="n"/>
+      <c r="D15" s="13" t="n">
+        <v>394</v>
+      </c>
+      <c r="E15" s="13" t="n">
+        <v>392</v>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G15" s="23" t="n">
         <v>388.3820277077359</v>
       </c>
@@ -7469,9 +7553,15 @@
       <c r="C16" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="13" t="n"/>
-      <c r="E16" s="13" t="n"/>
-      <c r="F16" s="13" t="n"/>
+      <c r="D16" s="13" t="n">
+        <v>394</v>
+      </c>
+      <c r="E16" s="13" t="n">
+        <v>392</v>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G16" s="23" t="n">
         <v>387.409894450538</v>
       </c>
@@ -7504,9 +7594,15 @@
       <c r="C17" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="13" t="n"/>
-      <c r="E17" s="13" t="n"/>
-      <c r="F17" s="13" t="n"/>
+      <c r="D17" s="13" t="n">
+        <v>394</v>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>392</v>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G17" s="23" t="n">
         <v>380.5761343495687</v>
       </c>
@@ -7539,9 +7635,15 @@
       <c r="C18" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D18" s="13" t="n"/>
-      <c r="E18" s="13" t="n"/>
-      <c r="F18" s="13" t="n"/>
+      <c r="D18" s="13" t="n">
+        <v>394.01</v>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>394</v>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>398.42</v>
+      </c>
       <c r="G18" s="23" t="n">
         <v>379.8197628231035</v>
       </c>
@@ -7574,9 +7676,15 @@
       <c r="C19" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D19" s="13" t="n"/>
-      <c r="E19" s="13" t="n"/>
-      <c r="F19" s="13" t="n"/>
+      <c r="D19" s="13" t="n">
+        <v>394.01</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>394</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>398.42</v>
+      </c>
       <c r="G19" s="23" t="n">
         <v>379.1034299842145</v>
       </c>
@@ -7609,9 +7717,15 @@
       <c r="C20" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D20" s="13" t="n"/>
-      <c r="E20" s="13" t="n"/>
-      <c r="F20" s="13" t="n"/>
+      <c r="D20" s="13" t="n">
+        <v>394.01</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>394</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>398.42</v>
+      </c>
       <c r="G20" s="23" t="n">
         <v>378.7110644951779</v>
       </c>
@@ -7644,9 +7758,15 @@
       <c r="C21" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D21" s="13" t="n"/>
-      <c r="E21" s="13" t="n"/>
-      <c r="F21" s="13" t="n"/>
+      <c r="D21" s="13" t="n">
+        <v>394.01</v>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>394</v>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>398.42</v>
+      </c>
       <c r="G21" s="23" t="n">
         <v>389.2115905914304</v>
       </c>
@@ -7679,9 +7799,15 @@
       <c r="C22" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="D22" s="13" t="n"/>
-      <c r="E22" s="13" t="n"/>
-      <c r="F22" s="13" t="n"/>
+      <c r="D22" s="13" t="n">
+        <v>397.13</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>396.85</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>409.39</v>
+      </c>
       <c r="G22" s="23" t="n">
         <v>394.1636938853383</v>
       </c>
@@ -7714,9 +7840,15 @@
       <c r="C23" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="D23" s="13" t="n"/>
-      <c r="E23" s="13" t="n"/>
-      <c r="F23" s="13" t="n"/>
+      <c r="D23" s="13" t="n">
+        <v>397.13</v>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>396.85</v>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>409.39</v>
+      </c>
       <c r="G23" s="23" t="n">
         <v>399.1891828011912</v>
       </c>
@@ -7749,9 +7881,15 @@
       <c r="C24" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
+      <c r="D24" s="13" t="n">
+        <v>397.13</v>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>396.85</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>409.39</v>
+      </c>
       <c r="G24" s="23" t="n">
         <v>407.3358657305317</v>
       </c>
@@ -7784,9 +7922,15 @@
       <c r="C25" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="D25" s="13" t="n"/>
-      <c r="E25" s="13" t="n"/>
-      <c r="F25" s="13" t="n"/>
+      <c r="D25" s="13" t="n">
+        <v>397.13</v>
+      </c>
+      <c r="E25" s="13" t="n">
+        <v>396.85</v>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>409.39</v>
+      </c>
       <c r="G25" s="23" t="n">
         <v>411.8435566100372</v>
       </c>
@@ -7819,9 +7963,15 @@
       <c r="C26" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="D26" s="13" t="n"/>
-      <c r="E26" s="13" t="n"/>
-      <c r="F26" s="13" t="n"/>
+      <c r="D26" s="13" t="n">
+        <v>390</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <v>389</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>408.89</v>
+      </c>
       <c r="G26" s="23" t="n">
         <v>409.7812245866</v>
       </c>
@@ -7854,9 +8004,15 @@
       <c r="C27" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="D27" s="13" t="n"/>
-      <c r="E27" s="13" t="n"/>
-      <c r="F27" s="13" t="n"/>
+      <c r="D27" s="13" t="n">
+        <v>390</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>389</v>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>408.89</v>
+      </c>
       <c r="G27" s="23" t="n">
         <v>405.6077617544083</v>
       </c>
@@ -7889,9 +8045,15 @@
       <c r="C28" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="D28" s="13" t="n"/>
-      <c r="E28" s="13" t="n"/>
-      <c r="F28" s="13" t="n"/>
+      <c r="D28" s="13" t="n">
+        <v>390</v>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>389</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>408.89</v>
+      </c>
       <c r="G28" s="23" t="n">
         <v>401.6933959962277</v>
       </c>
@@ -7924,9 +8086,15 @@
       <c r="C29" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="D29" s="13" t="n"/>
-      <c r="E29" s="13" t="n"/>
-      <c r="F29" s="13" t="n"/>
+      <c r="D29" s="13" t="n">
+        <v>390</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>389</v>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>408.89</v>
+      </c>
       <c r="G29" s="23" t="n">
         <v>394.2185160152247</v>
       </c>
@@ -7959,9 +8127,15 @@
       <c r="C30" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D30" s="13" t="n"/>
-      <c r="E30" s="13" t="n"/>
-      <c r="F30" s="13" t="n"/>
+      <c r="D30" s="13" t="n">
+        <v>372</v>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>371</v>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>378.77</v>
+      </c>
       <c r="G30" s="23" t="n">
         <v>378.621110105594</v>
       </c>
@@ -7994,9 +8168,15 @@
       <c r="C31" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D31" s="13" t="n"/>
-      <c r="E31" s="13" t="n"/>
-      <c r="F31" s="13" t="n"/>
+      <c r="D31" s="13" t="n">
+        <v>372</v>
+      </c>
+      <c r="E31" s="13" t="n">
+        <v>371</v>
+      </c>
+      <c r="F31" s="13" t="n">
+        <v>378.77</v>
+      </c>
       <c r="G31" s="23" t="n">
         <v>356.9704181029499</v>
       </c>
@@ -8029,9 +8209,15 @@
       <c r="C32" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D32" s="13" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n"/>
+      <c r="D32" s="13" t="n">
+        <v>372</v>
+      </c>
+      <c r="E32" s="13" t="n">
+        <v>371</v>
+      </c>
+      <c r="F32" s="13" t="n">
+        <v>378.77</v>
+      </c>
       <c r="G32" s="23" t="n">
         <v>345.7215427189589</v>
       </c>
@@ -8064,9 +8250,15 @@
       <c r="C33" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="D33" s="13" t="n"/>
-      <c r="E33" s="13" t="n"/>
-      <c r="F33" s="13" t="n"/>
+      <c r="D33" s="13" t="n">
+        <v>372</v>
+      </c>
+      <c r="E33" s="13" t="n">
+        <v>371</v>
+      </c>
+      <c r="F33" s="13" t="n">
+        <v>378.77</v>
+      </c>
       <c r="G33" s="23" t="n">
         <v>354.4917004344883</v>
       </c>
@@ -8099,9 +8291,15 @@
       <c r="C34" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="D34" s="13" t="n"/>
-      <c r="E34" s="13" t="n"/>
-      <c r="F34" s="13" t="n"/>
+      <c r="D34" s="13" t="n">
+        <v>360.52</v>
+      </c>
+      <c r="E34" s="13" t="n">
+        <v>348</v>
+      </c>
+      <c r="F34" s="13" t="n">
+        <v>365</v>
+      </c>
       <c r="G34" s="23" t="n">
         <v>342.3893237805008</v>
       </c>
@@ -8134,9 +8332,15 @@
       <c r="C35" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="D35" s="13" t="n"/>
-      <c r="E35" s="13" t="n"/>
-      <c r="F35" s="13" t="n"/>
+      <c r="D35" s="13" t="n">
+        <v>360.52</v>
+      </c>
+      <c r="E35" s="13" t="n">
+        <v>348</v>
+      </c>
+      <c r="F35" s="13" t="n">
+        <v>365</v>
+      </c>
       <c r="G35" s="23" t="n">
         <v>339.7778385635758</v>
       </c>
@@ -8169,9 +8373,15 @@
       <c r="C36" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="D36" s="13" t="n"/>
-      <c r="E36" s="13" t="n"/>
-      <c r="F36" s="13" t="n"/>
+      <c r="D36" s="13" t="n">
+        <v>360.52</v>
+      </c>
+      <c r="E36" s="13" t="n">
+        <v>348</v>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>365</v>
+      </c>
       <c r="G36" s="23" t="n">
         <v>307.9933511545871</v>
       </c>
@@ -8204,9 +8414,15 @@
       <c r="C37" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="D37" s="13" t="n"/>
-      <c r="E37" s="13" t="n"/>
-      <c r="F37" s="13" t="n"/>
+      <c r="D37" s="13" t="n">
+        <v>360.52</v>
+      </c>
+      <c r="E37" s="13" t="n">
+        <v>348</v>
+      </c>
+      <c r="F37" s="13" t="n">
+        <v>365</v>
+      </c>
       <c r="G37" s="23" t="n">
         <v>272.508478299232</v>
       </c>
@@ -8239,9 +8455,15 @@
       <c r="C38" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="D38" s="13" t="n"/>
-      <c r="E38" s="13" t="n"/>
-      <c r="F38" s="13" t="n"/>
+      <c r="D38" s="13" t="n">
+        <v>346.74</v>
+      </c>
+      <c r="E38" s="13" t="n">
+        <v>343.96</v>
+      </c>
+      <c r="F38" s="13" t="n">
+        <v>348</v>
+      </c>
       <c r="G38" s="23" t="n">
         <v>256.1254279138986</v>
       </c>
@@ -8274,9 +8496,15 @@
       <c r="C39" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="D39" s="13" t="n"/>
-      <c r="E39" s="13" t="n"/>
-      <c r="F39" s="13" t="n"/>
+      <c r="D39" s="13" t="n">
+        <v>346.74</v>
+      </c>
+      <c r="E39" s="13" t="n">
+        <v>343.96</v>
+      </c>
+      <c r="F39" s="13" t="n">
+        <v>348</v>
+      </c>
       <c r="G39" s="23" t="n">
         <v>251.5211580267692</v>
       </c>
@@ -8309,9 +8537,15 @@
       <c r="C40" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="D40" s="13" t="n"/>
-      <c r="E40" s="13" t="n"/>
-      <c r="F40" s="13" t="n"/>
+      <c r="D40" s="13" t="n">
+        <v>346.74</v>
+      </c>
+      <c r="E40" s="13" t="n">
+        <v>343.96</v>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>348</v>
+      </c>
       <c r="G40" s="23" t="n">
         <v>245.4161385929762</v>
       </c>
@@ -8344,9 +8578,15 @@
       <c r="C41" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="D41" s="13" t="n"/>
-      <c r="E41" s="13" t="n"/>
-      <c r="F41" s="13" t="n"/>
+      <c r="D41" s="13" t="n">
+        <v>346.74</v>
+      </c>
+      <c r="E41" s="13" t="n">
+        <v>343.96</v>
+      </c>
+      <c r="F41" s="13" t="n">
+        <v>348</v>
+      </c>
       <c r="G41" s="23" t="n">
         <v>234.9836597164605</v>
       </c>
@@ -8380,13 +8620,13 @@
         <v>11</v>
       </c>
       <c r="D42" s="13" t="n">
-        <v>338</v>
+        <v>337.35</v>
       </c>
       <c r="E42" s="13" t="n">
-        <v>338</v>
+        <v>290</v>
       </c>
       <c r="F42" s="13" t="n">
-        <v>338</v>
+        <v>338.99</v>
       </c>
       <c r="G42" s="23" t="n">
         <v>225.0104938130241</v>
@@ -8421,13 +8661,13 @@
         <v>11</v>
       </c>
       <c r="D43" s="13" t="n">
-        <v>338</v>
+        <v>337.35</v>
       </c>
       <c r="E43" s="13" t="n">
-        <v>338</v>
+        <v>290</v>
       </c>
       <c r="F43" s="13" t="n">
-        <v>338</v>
+        <v>338.99</v>
       </c>
       <c r="G43" s="23" t="n">
         <v>234.3726551498153</v>
@@ -8462,13 +8702,13 @@
         <v>11</v>
       </c>
       <c r="D44" s="13" t="n">
-        <v>338</v>
+        <v>337.35</v>
       </c>
       <c r="E44" s="13" t="n">
-        <v>338</v>
+        <v>290</v>
       </c>
       <c r="F44" s="13" t="n">
-        <v>338</v>
+        <v>338.99</v>
       </c>
       <c r="G44" s="23" t="n">
         <v>224.2613502713309</v>
@@ -8503,13 +8743,13 @@
         <v>11</v>
       </c>
       <c r="D45" s="13" t="n">
-        <v>338</v>
+        <v>337.35</v>
       </c>
       <c r="E45" s="13" t="n">
-        <v>338</v>
+        <v>290</v>
       </c>
       <c r="F45" s="13" t="n">
-        <v>338</v>
+        <v>338.99</v>
       </c>
       <c r="G45" s="23" t="n">
         <v>241.3663357474016</v>
@@ -8544,13 +8784,13 @@
         <v>12</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E46" s="13" t="n">
-        <v>362</v>
+        <v>353.06</v>
       </c>
       <c r="F46" s="13" t="n">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="G46" s="23" t="n">
         <v>249.1194754719694</v>
@@ -8585,13 +8825,13 @@
         <v>12</v>
       </c>
       <c r="D47" s="13" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E47" s="13" t="n">
-        <v>362</v>
+        <v>353.06</v>
       </c>
       <c r="F47" s="13" t="n">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="G47" s="23" t="n">
         <v>270.4525267792069</v>
@@ -8626,13 +8866,13 @@
         <v>12</v>
       </c>
       <c r="D48" s="13" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E48" s="13" t="n">
-        <v>362</v>
+        <v>353.06</v>
       </c>
       <c r="F48" s="13" t="n">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="G48" s="23" t="n">
         <v>267.4530185898701</v>
@@ -8667,13 +8907,13 @@
         <v>12</v>
       </c>
       <c r="D49" s="13" t="n">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="E49" s="13" t="n">
-        <v>362</v>
+        <v>353.06</v>
       </c>
       <c r="F49" s="13" t="n">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="G49" s="23" t="n">
         <v>254.887045698454</v>
@@ -8707,9 +8947,15 @@
       <c r="C50" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="D50" s="13" t="n"/>
-      <c r="E50" s="13" t="n"/>
-      <c r="F50" s="13" t="n"/>
+      <c r="D50" s="13" t="n">
+        <v>377</v>
+      </c>
+      <c r="E50" s="13" t="n">
+        <v>371.01</v>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>389</v>
+      </c>
       <c r="G50" s="23" t="n">
         <v>381.8318088643071</v>
       </c>
@@ -8742,9 +8988,15 @@
       <c r="C51" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="D51" s="13" t="n"/>
-      <c r="E51" s="13" t="n"/>
-      <c r="F51" s="13" t="n"/>
+      <c r="D51" s="13" t="n">
+        <v>377</v>
+      </c>
+      <c r="E51" s="13" t="n">
+        <v>371.01</v>
+      </c>
+      <c r="F51" s="13" t="n">
+        <v>389</v>
+      </c>
       <c r="G51" s="23" t="n">
         <v>314.7768884016766</v>
       </c>
@@ -8777,9 +9029,15 @@
       <c r="C52" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="D52" s="13" t="n"/>
-      <c r="E52" s="13" t="n"/>
-      <c r="F52" s="13" t="n"/>
+      <c r="D52" s="13" t="n">
+        <v>377</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>371.01</v>
+      </c>
+      <c r="F52" s="13" t="n">
+        <v>389</v>
+      </c>
       <c r="G52" s="23" t="n">
         <v>313.9932048382259</v>
       </c>
@@ -8812,9 +9070,15 @@
       <c r="C53" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="D53" s="13" t="n"/>
-      <c r="E53" s="13" t="n"/>
-      <c r="F53" s="13" t="n"/>
+      <c r="D53" s="13" t="n">
+        <v>377</v>
+      </c>
+      <c r="E53" s="13" t="n">
+        <v>371.01</v>
+      </c>
+      <c r="F53" s="13" t="n">
+        <v>389</v>
+      </c>
       <c r="G53" s="23" t="n">
         <v>312.1407129984934</v>
       </c>
@@ -8847,9 +9111,15 @@
       <c r="C54" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="D54" s="13" t="n"/>
-      <c r="E54" s="13" t="n"/>
-      <c r="F54" s="13" t="n"/>
+      <c r="D54" s="13" t="n">
+        <v>375</v>
+      </c>
+      <c r="E54" s="13" t="n">
+        <v>373.62</v>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>376</v>
+      </c>
       <c r="G54" s="23" t="n">
         <v>313.8166950261033</v>
       </c>
@@ -8882,9 +9152,15 @@
       <c r="C55" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="D55" s="13" t="n"/>
-      <c r="E55" s="13" t="n"/>
-      <c r="F55" s="13" t="n"/>
+      <c r="D55" s="13" t="n">
+        <v>375</v>
+      </c>
+      <c r="E55" s="13" t="n">
+        <v>373.62</v>
+      </c>
+      <c r="F55" s="13" t="n">
+        <v>376</v>
+      </c>
       <c r="G55" s="23" t="n">
         <v>313.4685474854437</v>
       </c>
@@ -8917,9 +9193,15 @@
       <c r="C56" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="D56" s="13" t="n"/>
-      <c r="E56" s="13" t="n"/>
-      <c r="F56" s="13" t="n"/>
+      <c r="D56" s="13" t="n">
+        <v>375</v>
+      </c>
+      <c r="E56" s="13" t="n">
+        <v>373.62</v>
+      </c>
+      <c r="F56" s="13" t="n">
+        <v>376</v>
+      </c>
       <c r="G56" s="23" t="n">
         <v>311.0154230362491</v>
       </c>
@@ -8952,9 +9234,15 @@
       <c r="C57" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="D57" s="13" t="n"/>
-      <c r="E57" s="13" t="n"/>
-      <c r="F57" s="13" t="n"/>
+      <c r="D57" s="13" t="n">
+        <v>375</v>
+      </c>
+      <c r="E57" s="13" t="n">
+        <v>373.62</v>
+      </c>
+      <c r="F57" s="13" t="n">
+        <v>376</v>
+      </c>
       <c r="G57" s="23" t="n">
         <v>267.1447724318896</v>
       </c>
@@ -8987,9 +9275,15 @@
       <c r="C58" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="D58" s="13" t="n"/>
-      <c r="E58" s="13" t="n"/>
-      <c r="F58" s="13" t="n"/>
+      <c r="D58" s="13" t="n">
+        <v>383</v>
+      </c>
+      <c r="E58" s="13" t="n">
+        <v>380.02</v>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>398.97</v>
+      </c>
       <c r="G58" s="23" t="n">
         <v>268.7042428907612</v>
       </c>
@@ -9022,9 +9316,15 @@
       <c r="C59" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="D59" s="13" t="n"/>
-      <c r="E59" s="13" t="n"/>
-      <c r="F59" s="13" t="n"/>
+      <c r="D59" s="13" t="n">
+        <v>383</v>
+      </c>
+      <c r="E59" s="13" t="n">
+        <v>380.02</v>
+      </c>
+      <c r="F59" s="13" t="n">
+        <v>398.97</v>
+      </c>
       <c r="G59" s="23" t="n">
         <v>297.9924735203632</v>
       </c>
@@ -9057,9 +9357,15 @@
       <c r="C60" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="D60" s="13" t="n"/>
-      <c r="E60" s="13" t="n"/>
-      <c r="F60" s="13" t="n"/>
+      <c r="D60" s="13" t="n">
+        <v>383</v>
+      </c>
+      <c r="E60" s="13" t="n">
+        <v>380.02</v>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>398.97</v>
+      </c>
       <c r="G60" s="23" t="n">
         <v>310.2891840945099</v>
       </c>
@@ -9092,9 +9398,15 @@
       <c r="C61" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="D61" s="13" t="n"/>
-      <c r="E61" s="13" t="n"/>
-      <c r="F61" s="13" t="n"/>
+      <c r="D61" s="13" t="n">
+        <v>383</v>
+      </c>
+      <c r="E61" s="13" t="n">
+        <v>380.02</v>
+      </c>
+      <c r="F61" s="13" t="n">
+        <v>398.97</v>
+      </c>
       <c r="G61" s="23" t="n">
         <v>294.2460800684168</v>
       </c>
@@ -9127,9 +9439,15 @@
       <c r="C62" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="D62" s="13" t="n"/>
-      <c r="E62" s="13" t="n"/>
-      <c r="F62" s="13" t="n"/>
+      <c r="D62" s="13" t="n">
+        <v>395</v>
+      </c>
+      <c r="E62" s="13" t="n">
+        <v>393.3</v>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G62" s="23" t="n">
         <v>276.6998654803334</v>
       </c>
@@ -9162,9 +9480,15 @@
       <c r="C63" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="D63" s="13" t="n"/>
-      <c r="E63" s="13" t="n"/>
-      <c r="F63" s="13" t="n"/>
+      <c r="D63" s="13" t="n">
+        <v>395</v>
+      </c>
+      <c r="E63" s="13" t="n">
+        <v>393.3</v>
+      </c>
+      <c r="F63" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G63" s="23" t="n">
         <v>291.1104298825689</v>
       </c>
@@ -9197,9 +9521,15 @@
       <c r="C64" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="D64" s="13" t="n"/>
-      <c r="E64" s="13" t="n"/>
-      <c r="F64" s="13" t="n"/>
+      <c r="D64" s="13" t="n">
+        <v>395</v>
+      </c>
+      <c r="E64" s="13" t="n">
+        <v>393.3</v>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G64" s="23" t="n">
         <v>300.1730438828101</v>
       </c>
@@ -9232,9 +9562,15 @@
       <c r="C65" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="D65" s="13" t="n"/>
-      <c r="E65" s="13" t="n"/>
-      <c r="F65" s="13" t="n"/>
+      <c r="D65" s="13" t="n">
+        <v>395</v>
+      </c>
+      <c r="E65" s="13" t="n">
+        <v>393.3</v>
+      </c>
+      <c r="F65" s="13" t="n">
+        <v>405</v>
+      </c>
       <c r="G65" s="23" t="n">
         <v>309.2401327225067</v>
       </c>
@@ -9267,9 +9603,15 @@
       <c r="C66" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D66" s="13" t="n"/>
-      <c r="E66" s="13" t="n"/>
-      <c r="F66" s="13" t="n"/>
+      <c r="D66" s="13" t="n">
+        <v>415.98</v>
+      </c>
+      <c r="E66" s="13" t="n">
+        <v>414</v>
+      </c>
+      <c r="F66" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G66" s="23" t="n">
         <v>333.4975608766179</v>
       </c>
@@ -9302,9 +9644,15 @@
       <c r="C67" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D67" s="13" t="n"/>
-      <c r="E67" s="13" t="n"/>
-      <c r="F67" s="13" t="n"/>
+      <c r="D67" s="13" t="n">
+        <v>415.98</v>
+      </c>
+      <c r="E67" s="13" t="n">
+        <v>414</v>
+      </c>
+      <c r="F67" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G67" s="23" t="n">
         <v>353.8508414579547</v>
       </c>
@@ -9337,9 +9685,15 @@
       <c r="C68" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D68" s="13" t="n"/>
-      <c r="E68" s="13" t="n"/>
-      <c r="F68" s="13" t="n"/>
+      <c r="D68" s="13" t="n">
+        <v>415.98</v>
+      </c>
+      <c r="E68" s="13" t="n">
+        <v>414</v>
+      </c>
+      <c r="F68" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G68" s="23" t="n">
         <v>388.8799529633367</v>
       </c>
@@ -9372,9 +9726,15 @@
       <c r="C69" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="D69" s="13" t="n"/>
-      <c r="E69" s="13" t="n"/>
-      <c r="F69" s="13" t="n"/>
+      <c r="D69" s="13" t="n">
+        <v>415.98</v>
+      </c>
+      <c r="E69" s="13" t="n">
+        <v>414</v>
+      </c>
+      <c r="F69" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G69" s="23" t="n">
         <v>406.5605973878581</v>
       </c>
@@ -9407,9 +9767,15 @@
       <c r="C70" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="D70" s="13" t="n"/>
-      <c r="E70" s="13" t="n"/>
-      <c r="F70" s="13" t="n"/>
+      <c r="D70" s="13" t="n">
+        <v>420</v>
+      </c>
+      <c r="E70" s="13" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="F70" s="13" t="n">
+        <v>433.99</v>
+      </c>
       <c r="G70" s="23" t="n">
         <v>392.3608642722835</v>
       </c>
@@ -9442,9 +9808,15 @@
       <c r="C71" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="D71" s="13" t="n"/>
-      <c r="E71" s="13" t="n"/>
-      <c r="F71" s="13" t="n"/>
+      <c r="D71" s="13" t="n">
+        <v>420</v>
+      </c>
+      <c r="E71" s="13" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="F71" s="13" t="n">
+        <v>433.99</v>
+      </c>
       <c r="G71" s="23" t="n">
         <v>405.2711913883359</v>
       </c>
@@ -9477,9 +9849,15 @@
       <c r="C72" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="D72" s="13" t="n"/>
-      <c r="E72" s="13" t="n"/>
-      <c r="F72" s="13" t="n"/>
+      <c r="D72" s="13" t="n">
+        <v>420</v>
+      </c>
+      <c r="E72" s="13" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="F72" s="13" t="n">
+        <v>433.99</v>
+      </c>
       <c r="G72" s="23" t="n">
         <v>406.6868975139006</v>
       </c>
@@ -9512,9 +9890,15 @@
       <c r="C73" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="D73" s="13" t="n"/>
-      <c r="E73" s="13" t="n"/>
-      <c r="F73" s="13" t="n"/>
+      <c r="D73" s="13" t="n">
+        <v>420</v>
+      </c>
+      <c r="E73" s="13" t="n">
+        <v>419.1</v>
+      </c>
+      <c r="F73" s="13" t="n">
+        <v>433.99</v>
+      </c>
       <c r="G73" s="23" t="n">
         <v>406.3892922830289</v>
       </c>
@@ -9547,9 +9931,15 @@
       <c r="C74" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="D74" s="13" t="n"/>
-      <c r="E74" s="13" t="n"/>
-      <c r="F74" s="13" t="n"/>
+      <c r="D74" s="13" t="n">
+        <v>419</v>
+      </c>
+      <c r="E74" s="13" t="n">
+        <v>416.01</v>
+      </c>
+      <c r="F74" s="13" t="n">
+        <v>423</v>
+      </c>
       <c r="G74" s="23" t="n">
         <v>397.4337824925005</v>
       </c>
@@ -9582,9 +9972,15 @@
       <c r="C75" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="D75" s="13" t="n"/>
-      <c r="E75" s="13" t="n"/>
-      <c r="F75" s="13" t="n"/>
+      <c r="D75" s="13" t="n">
+        <v>419</v>
+      </c>
+      <c r="E75" s="13" t="n">
+        <v>416.01</v>
+      </c>
+      <c r="F75" s="13" t="n">
+        <v>423</v>
+      </c>
       <c r="G75" s="23" t="n">
         <v>398.2680614545064</v>
       </c>
@@ -9617,9 +10013,15 @@
       <c r="C76" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="D76" s="13" t="n"/>
-      <c r="E76" s="13" t="n"/>
-      <c r="F76" s="13" t="n"/>
+      <c r="D76" s="13" t="n">
+        <v>419</v>
+      </c>
+      <c r="E76" s="13" t="n">
+        <v>416.01</v>
+      </c>
+      <c r="F76" s="13" t="n">
+        <v>423</v>
+      </c>
       <c r="G76" s="23" t="n">
         <v>402.7605771261515</v>
       </c>
@@ -9652,9 +10054,15 @@
       <c r="C77" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="D77" s="13" t="n"/>
-      <c r="E77" s="13" t="n"/>
-      <c r="F77" s="13" t="n"/>
+      <c r="D77" s="13" t="n">
+        <v>419</v>
+      </c>
+      <c r="E77" s="13" t="n">
+        <v>416.01</v>
+      </c>
+      <c r="F77" s="13" t="n">
+        <v>423</v>
+      </c>
       <c r="G77" s="23" t="n">
         <v>406.124318557978</v>
       </c>
@@ -9687,9 +10095,15 @@
       <c r="C78" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="D78" s="13" t="n"/>
-      <c r="E78" s="13" t="n"/>
-      <c r="F78" s="13" t="n"/>
+      <c r="D78" s="13" t="n">
+        <v>417.13</v>
+      </c>
+      <c r="E78" s="13" t="n">
+        <v>415</v>
+      </c>
+      <c r="F78" s="13" t="n">
+        <v>419</v>
+      </c>
       <c r="G78" s="23" t="n">
         <v>398.9981315426662</v>
       </c>
@@ -9722,9 +10136,15 @@
       <c r="C79" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="D79" s="13" t="n"/>
-      <c r="E79" s="13" t="n"/>
-      <c r="F79" s="13" t="n"/>
+      <c r="D79" s="13" t="n">
+        <v>417.13</v>
+      </c>
+      <c r="E79" s="13" t="n">
+        <v>415</v>
+      </c>
+      <c r="F79" s="13" t="n">
+        <v>419</v>
+      </c>
       <c r="G79" s="23" t="n">
         <v>399.855617713881</v>
       </c>
@@ -9757,9 +10177,15 @@
       <c r="C80" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="D80" s="13" t="n"/>
-      <c r="E80" s="13" t="n"/>
-      <c r="F80" s="13" t="n"/>
+      <c r="D80" s="13" t="n">
+        <v>417.13</v>
+      </c>
+      <c r="E80" s="13" t="n">
+        <v>415</v>
+      </c>
+      <c r="F80" s="13" t="n">
+        <v>419</v>
+      </c>
       <c r="G80" s="23" t="n">
         <v>392.9702578812335</v>
       </c>
@@ -9792,9 +10218,15 @@
       <c r="C81" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="D81" s="13" t="n"/>
-      <c r="E81" s="13" t="n"/>
-      <c r="F81" s="13" t="n"/>
+      <c r="D81" s="13" t="n">
+        <v>417.13</v>
+      </c>
+      <c r="E81" s="13" t="n">
+        <v>415</v>
+      </c>
+      <c r="F81" s="13" t="n">
+        <v>419</v>
+      </c>
       <c r="G81" s="23" t="n">
         <v>388.3126803086009</v>
       </c>
@@ -9827,9 +10259,15 @@
       <c r="C82" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="D82" s="13" t="n"/>
-      <c r="E82" s="13" t="n"/>
-      <c r="F82" s="13" t="n"/>
+      <c r="D82" s="13" t="n">
+        <v>411</v>
+      </c>
+      <c r="E82" s="13" t="n">
+        <v>409</v>
+      </c>
+      <c r="F82" s="13" t="n">
+        <v>414</v>
+      </c>
       <c r="G82" s="23" t="n">
         <v>386.0087959262887</v>
       </c>
@@ -9862,9 +10300,15 @@
       <c r="C83" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="D83" s="13" t="n"/>
-      <c r="E83" s="13" t="n"/>
-      <c r="F83" s="13" t="n"/>
+      <c r="D83" s="13" t="n">
+        <v>411</v>
+      </c>
+      <c r="E83" s="13" t="n">
+        <v>409</v>
+      </c>
+      <c r="F83" s="13" t="n">
+        <v>414</v>
+      </c>
       <c r="G83" s="23" t="n">
         <v>384.7143781847317</v>
       </c>
@@ -9897,9 +10341,15 @@
       <c r="C84" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="D84" s="13" t="n"/>
-      <c r="E84" s="13" t="n"/>
-      <c r="F84" s="13" t="n"/>
+      <c r="D84" s="13" t="n">
+        <v>411</v>
+      </c>
+      <c r="E84" s="13" t="n">
+        <v>409</v>
+      </c>
+      <c r="F84" s="13" t="n">
+        <v>414</v>
+      </c>
       <c r="G84" s="23" t="n">
         <v>389.4658725621233</v>
       </c>
@@ -9932,9 +10382,15 @@
       <c r="C85" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="D85" s="13" t="n"/>
-      <c r="E85" s="13" t="n"/>
-      <c r="F85" s="13" t="n"/>
+      <c r="D85" s="13" t="n">
+        <v>411</v>
+      </c>
+      <c r="E85" s="13" t="n">
+        <v>409</v>
+      </c>
+      <c r="F85" s="13" t="n">
+        <v>414</v>
+      </c>
       <c r="G85" s="23" t="n">
         <v>396.9908278773645</v>
       </c>
@@ -9967,9 +10423,15 @@
       <c r="C86" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="D86" s="13" t="n"/>
-      <c r="E86" s="13" t="n"/>
-      <c r="F86" s="13" t="n"/>
+      <c r="D86" s="13" t="n">
+        <v>413</v>
+      </c>
+      <c r="E86" s="13" t="n">
+        <v>407</v>
+      </c>
+      <c r="F86" s="13" t="n">
+        <v>415</v>
+      </c>
       <c r="G86" s="23" t="n">
         <v>392.9437092731382</v>
       </c>
@@ -10002,9 +10464,15 @@
       <c r="C87" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="D87" s="13" t="n"/>
-      <c r="E87" s="13" t="n"/>
-      <c r="F87" s="13" t="n"/>
+      <c r="D87" s="13" t="n">
+        <v>413</v>
+      </c>
+      <c r="E87" s="13" t="n">
+        <v>407</v>
+      </c>
+      <c r="F87" s="13" t="n">
+        <v>415</v>
+      </c>
       <c r="G87" s="23" t="n">
         <v>395.396133405918</v>
       </c>
@@ -10037,9 +10505,15 @@
       <c r="C88" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="D88" s="13" t="n"/>
-      <c r="E88" s="13" t="n"/>
-      <c r="F88" s="13" t="n"/>
+      <c r="D88" s="13" t="n">
+        <v>413</v>
+      </c>
+      <c r="E88" s="13" t="n">
+        <v>407</v>
+      </c>
+      <c r="F88" s="13" t="n">
+        <v>415</v>
+      </c>
       <c r="G88" s="23" t="n">
         <v>390.1798734374863</v>
       </c>
@@ -10072,9 +10546,15 @@
       <c r="C89" s="3" t="n">
         <v>22</v>
       </c>
-      <c r="D89" s="13" t="n"/>
-      <c r="E89" s="13" t="n"/>
-      <c r="F89" s="13" t="n"/>
+      <c r="D89" s="13" t="n">
+        <v>413</v>
+      </c>
+      <c r="E89" s="13" t="n">
+        <v>407</v>
+      </c>
+      <c r="F89" s="13" t="n">
+        <v>415</v>
+      </c>
       <c r="G89" s="23" t="n">
         <v>388.0591390837571</v>
       </c>
@@ -10107,9 +10587,15 @@
       <c r="C90" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="D90" s="13" t="n"/>
-      <c r="E90" s="13" t="n"/>
-      <c r="F90" s="13" t="n"/>
+      <c r="D90" s="13" t="n">
+        <v>415.63</v>
+      </c>
+      <c r="E90" s="13" t="n">
+        <v>412.01</v>
+      </c>
+      <c r="F90" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G90" s="23" t="n">
         <v>384.3143502118286</v>
       </c>
@@ -10142,9 +10628,15 @@
       <c r="C91" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="D91" s="13" t="n"/>
-      <c r="E91" s="13" t="n"/>
-      <c r="F91" s="13" t="n"/>
+      <c r="D91" s="13" t="n">
+        <v>415.63</v>
+      </c>
+      <c r="E91" s="13" t="n">
+        <v>412.01</v>
+      </c>
+      <c r="F91" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G91" s="23" t="n">
         <v>388.7586350623399</v>
       </c>
@@ -10177,9 +10669,15 @@
       <c r="C92" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="D92" s="13" t="n"/>
-      <c r="E92" s="13" t="n"/>
-      <c r="F92" s="13" t="n"/>
+      <c r="D92" s="13" t="n">
+        <v>415.63</v>
+      </c>
+      <c r="E92" s="13" t="n">
+        <v>412.01</v>
+      </c>
+      <c r="F92" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G92" s="23" t="n">
         <v>398.6155222030513</v>
       </c>
@@ -10212,9 +10710,15 @@
       <c r="C93" s="3" t="n">
         <v>23</v>
       </c>
-      <c r="D93" s="13" t="n"/>
-      <c r="E93" s="13" t="n"/>
-      <c r="F93" s="13" t="n"/>
+      <c r="D93" s="13" t="n">
+        <v>415.63</v>
+      </c>
+      <c r="E93" s="13" t="n">
+        <v>412.01</v>
+      </c>
+      <c r="F93" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G93" s="23" t="n">
         <v>409.2970433338114</v>
       </c>
@@ -10247,9 +10751,15 @@
       <c r="C94" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="D94" s="13" t="n"/>
-      <c r="E94" s="13" t="n"/>
-      <c r="F94" s="13" t="n"/>
+      <c r="D94" s="13" t="n">
+        <v>415</v>
+      </c>
+      <c r="E94" s="13" t="n">
+        <v>410</v>
+      </c>
+      <c r="F94" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G94" s="23" t="n">
         <v>426.6199635572671</v>
       </c>
@@ -10282,9 +10792,15 @@
       <c r="C95" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="D95" s="13" t="n"/>
-      <c r="E95" s="13" t="n"/>
-      <c r="F95" s="13" t="n"/>
+      <c r="D95" s="13" t="n">
+        <v>415</v>
+      </c>
+      <c r="E95" s="13" t="n">
+        <v>410</v>
+      </c>
+      <c r="F95" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G95" s="23" t="n">
         <v>411.6626057647354</v>
       </c>
@@ -10317,9 +10833,15 @@
       <c r="C96" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="D96" s="13" t="n"/>
-      <c r="E96" s="13" t="n"/>
-      <c r="F96" s="13" t="n"/>
+      <c r="D96" s="13" t="n">
+        <v>415</v>
+      </c>
+      <c r="E96" s="13" t="n">
+        <v>410</v>
+      </c>
+      <c r="F96" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G96" s="23" t="n">
         <v>406.3261644419341</v>
       </c>
@@ -10354,9 +10876,15 @@
       <c r="C97" s="3" t="n">
         <v>24</v>
       </c>
-      <c r="D97" s="13" t="n"/>
-      <c r="E97" s="13" t="n"/>
-      <c r="F97" s="13" t="n"/>
+      <c r="D97" s="13" t="n">
+        <v>415</v>
+      </c>
+      <c r="E97" s="13" t="n">
+        <v>410</v>
+      </c>
+      <c r="F97" s="13" t="n">
+        <v>420</v>
+      </c>
       <c r="G97" s="23" t="n">
         <v>408.3785508182123</v>
       </c>

</xml_diff>